<commit_message>
Update DraxosMobile character systems rework
</commit_message>
<xml_diff>
--- a/Projetos/draxos-mobile/docs/economy/generated/draxos_mobile_economy_simulator.xlsx
+++ b/Projetos/draxos-mobile/docs/economy/generated/draxos_mobile_economy_simulator.xlsx
@@ -912,7 +912,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Upgrade de varinha e spells</t>
+          <t>Upgrade de Instrumento Ritual e spells</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -976,7 +976,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Upgrade de pets</t>
+          <t>Upgrade de Familiares</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Upgrade de passivas</t>
+          <t>Upgrade de Doutrinas</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1040,7 +1040,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Qualidade e crafting da varinha</t>
+          <t>Qualidade e crafting do Instrumento Ritual</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">

</xml_diff>